<commit_message>
Rathgeb: geprüfte Namen und Bio-Angaben der Teilbetriebe (Knospe-Zertifikate, Ellikon ehem. Kellermann, BioFresh)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQ5MKVLWHBWiVwJge7L58K
</commit_message>
<xml_diff>
--- a/output/Feldkarte_Flaechen_4_Betriebe.xlsx
+++ b/output/Feldkarte_Flaechen_4_Betriebe.xlsx
@@ -500,7 +500,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Betriebsnummern: Imhof ZH0197/ 1/  1 + ZH0197/ 1/702 · Beerstecher ZH0191/ 1/ 55 · Gerber ZH0172/ 1/700 (Zwei Firmen unter einer Betriebsnummer; aufgeteilt nach den amtlichen Produktionsstätten) · Rathgeb ZH0042/ 1/850 + TG39621 (Drei Teile unter zwei Betriebsnummern; aufgeteilt nach den amtlichen Produktionsstätten)</t>
+          <t>Betriebsnummern: Imhof ZH0197/ 1/  1 + ZH0197/ 1/702 · Beerstecher ZH0191/ 1/ 55 · Gerber ZH0172/ 1/700 (Zwei Firmen unter einer Betriebsnummer; aufgeteilt nach den amtlichen Produktionsstätten) · Rathgeb ZH0042/ 1/850 + TG39621 (Unternehmensgruppe: drei Teile unter zwei Betriebsnummern, getrennt nach amtlicher Produktionsstätte)</t>
         </is>
       </c>
     </row>
@@ -955,14 +955,14 @@
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Bio (Knospe); Flächen als Bioproduktion gemeldet</t>
+          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Flächen als Bioproduktion gemeldet</t>
+          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Flächen als Bioproduktion gemeldet</t>
+          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
         </is>
       </c>
     </row>
@@ -41914,7 +41914,7 @@
       </c>
       <c r="M654" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N654" s="4" t="inlineStr">
@@ -42042,7 +42042,7 @@
       </c>
       <c r="M656" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N656" s="4" t="inlineStr">
@@ -42106,7 +42106,7 @@
       </c>
       <c r="M657" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N657" s="4" t="inlineStr">
@@ -42170,7 +42170,7 @@
       </c>
       <c r="M658" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N658" s="4" t="inlineStr">
@@ -42234,7 +42234,7 @@
       </c>
       <c r="M659" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N659" s="4" t="inlineStr">
@@ -42298,7 +42298,7 @@
       </c>
       <c r="M660" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N660" s="4" t="inlineStr">
@@ -42362,7 +42362,7 @@
       </c>
       <c r="M661" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N661" s="4" t="inlineStr">
@@ -42426,7 +42426,7 @@
       </c>
       <c r="M662" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N662" s="4" t="inlineStr">
@@ -42490,7 +42490,7 @@
       </c>
       <c r="M663" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N663" s="4" t="inlineStr">
@@ -42554,7 +42554,7 @@
       </c>
       <c r="M664" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N664" s="4" t="inlineStr">
@@ -42618,7 +42618,7 @@
       </c>
       <c r="M665" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N665" s="4" t="inlineStr">
@@ -42682,7 +42682,7 @@
       </c>
       <c r="M666" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N666" s="4" t="inlineStr">
@@ -42810,7 +42810,7 @@
       </c>
       <c r="M668" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N668" s="4" t="inlineStr">
@@ -42874,7 +42874,7 @@
       </c>
       <c r="M669" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N669" s="4" t="inlineStr">
@@ -43258,7 +43258,7 @@
       </c>
       <c r="M675" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N675" s="4" t="inlineStr">
@@ -43322,7 +43322,7 @@
       </c>
       <c r="M676" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N676" s="4" t="inlineStr">
@@ -43386,7 +43386,7 @@
       </c>
       <c r="M677" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N677" s="4" t="inlineStr">
@@ -43578,7 +43578,7 @@
       </c>
       <c r="M680" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N680" s="4" t="inlineStr">
@@ -43706,7 +43706,7 @@
       </c>
       <c r="M682" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N682" s="4" t="inlineStr">
@@ -43962,7 +43962,7 @@
       </c>
       <c r="M686" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N686" s="4" t="inlineStr">
@@ -44218,7 +44218,7 @@
       </c>
       <c r="M690" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N690" s="4" t="inlineStr">
@@ -44282,7 +44282,7 @@
       </c>
       <c r="M691" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N691" s="4" t="inlineStr">
@@ -44474,7 +44474,7 @@
       </c>
       <c r="M694" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N694" s="4" t="inlineStr">
@@ -44794,7 +44794,7 @@
       </c>
       <c r="M699" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N699" s="4" t="inlineStr">
@@ -44986,7 +44986,7 @@
       </c>
       <c r="M702" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N702" s="4" t="inlineStr">
@@ -45242,7 +45242,7 @@
       </c>
       <c r="M706" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N706" s="4" t="inlineStr">
@@ -45562,7 +45562,7 @@
       </c>
       <c r="M711" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N711" s="4" t="inlineStr">
@@ -45882,7 +45882,7 @@
       </c>
       <c r="M716" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N716" s="4" t="inlineStr">
@@ -46010,7 +46010,7 @@
       </c>
       <c r="M718" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N718" s="4" t="inlineStr">
@@ -46266,7 +46266,7 @@
       </c>
       <c r="M722" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N722" s="4" t="inlineStr">
@@ -46330,7 +46330,7 @@
       </c>
       <c r="M723" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N723" s="4" t="inlineStr">
@@ -46394,7 +46394,7 @@
       </c>
       <c r="M724" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N724" s="4" t="inlineStr">
@@ -46586,7 +46586,7 @@
       </c>
       <c r="M727" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N727" s="4" t="inlineStr">
@@ -46714,7 +46714,7 @@
       </c>
       <c r="M729" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N729" s="4" t="inlineStr">
@@ -46970,7 +46970,7 @@
       </c>
       <c r="M733" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N733" s="4" t="inlineStr">
@@ -47034,7 +47034,7 @@
       </c>
       <c r="M734" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N734" s="4" t="inlineStr">
@@ -47162,7 +47162,7 @@
       </c>
       <c r="M736" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N736" s="4" t="inlineStr">
@@ -47354,7 +47354,7 @@
       </c>
       <c r="M739" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N739" s="4" t="inlineStr">
@@ -47546,7 +47546,7 @@
       </c>
       <c r="M742" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N742" s="4" t="inlineStr">
@@ -47674,7 +47674,7 @@
       </c>
       <c r="M744" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N744" s="4" t="inlineStr">
@@ -47866,7 +47866,7 @@
       </c>
       <c r="M747" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N747" s="4" t="inlineStr">
@@ -48314,7 +48314,7 @@
       </c>
       <c r="M754" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N754" s="4" t="inlineStr">
@@ -48378,7 +48378,7 @@
       </c>
       <c r="M755" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N755" s="4" t="inlineStr">
@@ -48442,7 +48442,7 @@
       </c>
       <c r="M756" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N756" s="4" t="inlineStr">
@@ -48506,7 +48506,7 @@
       </c>
       <c r="M757" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N757" s="4" t="inlineStr">
@@ -48570,7 +48570,7 @@
       </c>
       <c r="M758" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N758" s="4" t="inlineStr">
@@ -48634,7 +48634,7 @@
       </c>
       <c r="M759" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N759" s="4" t="inlineStr">
@@ -48698,7 +48698,7 @@
       </c>
       <c r="M760" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N760" s="4" t="inlineStr">
@@ -48762,7 +48762,7 @@
       </c>
       <c r="M761" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N761" s="4" t="inlineStr">
@@ -48890,7 +48890,7 @@
       </c>
       <c r="M763" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N763" s="4" t="inlineStr">
@@ -49402,7 +49402,7 @@
       </c>
       <c r="M771" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N771" s="4" t="inlineStr">
@@ -49466,7 +49466,7 @@
       </c>
       <c r="M772" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N772" s="4" t="inlineStr">
@@ -49530,7 +49530,7 @@
       </c>
       <c r="M773" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N773" s="4" t="inlineStr">
@@ -49658,7 +49658,7 @@
       </c>
       <c r="M775" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N775" s="4" t="inlineStr">
@@ -49786,7 +49786,7 @@
       </c>
       <c r="M777" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N777" s="4" t="inlineStr">
@@ -49914,7 +49914,7 @@
       </c>
       <c r="M779" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N779" s="4" t="inlineStr">
@@ -50042,7 +50042,7 @@
       </c>
       <c r="M781" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N781" s="4" t="inlineStr">
@@ -50170,7 +50170,7 @@
       </c>
       <c r="M783" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N783" s="4" t="inlineStr">
@@ -50362,7 +50362,7 @@
       </c>
       <c r="M786" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N786" s="4" t="inlineStr">
@@ -50426,7 +50426,7 @@
       </c>
       <c r="M787" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N787" s="4" t="inlineStr">
@@ -50490,7 +50490,7 @@
       </c>
       <c r="M788" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N788" s="4" t="inlineStr">
@@ -50554,7 +50554,7 @@
       </c>
       <c r="M789" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N789" s="4" t="inlineStr">
@@ -50874,7 +50874,7 @@
       </c>
       <c r="M794" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N794" s="4" t="inlineStr">
@@ -51130,7 +51130,7 @@
       </c>
       <c r="M798" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N798" s="4" t="inlineStr">
@@ -51194,7 +51194,7 @@
       </c>
       <c r="M799" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N799" s="4" t="inlineStr">
@@ -51258,7 +51258,7 @@
       </c>
       <c r="M800" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N800" s="4" t="inlineStr">
@@ -51322,7 +51322,7 @@
       </c>
       <c r="M801" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N801" s="4" t="inlineStr">
@@ -51642,7 +51642,7 @@
       </c>
       <c r="M806" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N806" s="4" t="inlineStr">
@@ -51770,7 +51770,7 @@
       </c>
       <c r="M808" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N808" s="4" t="inlineStr">
@@ -52026,7 +52026,7 @@
       </c>
       <c r="M812" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N812" s="4" t="inlineStr">
@@ -52282,7 +52282,7 @@
       </c>
       <c r="M816" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N816" s="4" t="inlineStr">
@@ -52474,7 +52474,7 @@
       </c>
       <c r="M819" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N819" s="4" t="inlineStr">
@@ -52666,7 +52666,7 @@
       </c>
       <c r="M822" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N822" s="4" t="inlineStr">
@@ -52986,7 +52986,7 @@
       </c>
       <c r="M827" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N827" s="4" t="inlineStr">
@@ -53050,7 +53050,7 @@
       </c>
       <c r="M828" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N828" s="4" t="inlineStr">
@@ -53114,7 +53114,7 @@
       </c>
       <c r="M829" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N829" s="4" t="inlineStr">
@@ -53242,7 +53242,7 @@
       </c>
       <c r="M831" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N831" s="4" t="inlineStr">
@@ -53306,7 +53306,7 @@
       </c>
       <c r="M832" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N832" s="4" t="inlineStr">
@@ -53370,7 +53370,7 @@
       </c>
       <c r="M833" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N833" s="4" t="inlineStr">
@@ -53434,7 +53434,7 @@
       </c>
       <c r="M834" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N834" s="4" t="inlineStr">
@@ -53818,7 +53818,7 @@
       </c>
       <c r="M840" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N840" s="4" t="inlineStr">
@@ -54202,7 +54202,7 @@
       </c>
       <c r="M846" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N846" s="4" t="inlineStr">
@@ -54266,7 +54266,7 @@
       </c>
       <c r="M847" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N847" s="4" t="inlineStr">
@@ -54330,7 +54330,7 @@
       </c>
       <c r="M848" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N848" s="4" t="inlineStr">
@@ -54394,7 +54394,7 @@
       </c>
       <c r="M849" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N849" s="4" t="inlineStr">
@@ -54522,7 +54522,7 @@
       </c>
       <c r="M851" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N851" s="4" t="inlineStr">
@@ -54586,7 +54586,7 @@
       </c>
       <c r="M852" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N852" s="4" t="inlineStr">
@@ -54650,7 +54650,7 @@
       </c>
       <c r="M853" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N853" s="4" t="inlineStr">
@@ -54778,7 +54778,7 @@
       </c>
       <c r="M855" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N855" s="4" t="inlineStr">
@@ -54906,7 +54906,7 @@
       </c>
       <c r="M857" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N857" s="4" t="inlineStr">
@@ -54970,7 +54970,7 @@
       </c>
       <c r="M858" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N858" s="4" t="inlineStr">
@@ -55158,7 +55158,7 @@
       </c>
       <c r="M861" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N861" s="4" t="inlineStr">
@@ -55350,7 +55350,7 @@
       </c>
       <c r="M864" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N864" s="4" t="inlineStr">
@@ -55414,7 +55414,7 @@
       </c>
       <c r="M865" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N865" s="4" t="inlineStr">
@@ -55478,7 +55478,7 @@
       </c>
       <c r="M866" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N866" s="4" t="inlineStr">
@@ -55542,7 +55542,7 @@
       </c>
       <c r="M867" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N867" s="4" t="inlineStr">
@@ -55606,7 +55606,7 @@
       </c>
       <c r="M868" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N868" s="4" t="inlineStr">
@@ -55862,7 +55862,7 @@
       </c>
       <c r="M872" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N872" s="4" t="inlineStr">
@@ -55926,7 +55926,7 @@
       </c>
       <c r="M873" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N873" s="4" t="inlineStr">
@@ -56054,7 +56054,7 @@
       </c>
       <c r="M875" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N875" s="4" t="inlineStr">
@@ -56118,7 +56118,7 @@
       </c>
       <c r="M876" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N876" s="4" t="inlineStr">
@@ -56310,7 +56310,7 @@
       </c>
       <c r="M879" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N879" s="4" t="inlineStr">
@@ -56374,7 +56374,7 @@
       </c>
       <c r="M880" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N880" s="4" t="inlineStr">
@@ -56434,7 +56434,7 @@
       </c>
       <c r="M881" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N881" s="4" t="inlineStr">
@@ -56498,7 +56498,7 @@
       </c>
       <c r="M882" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N882" s="4" t="inlineStr">
@@ -56562,7 +56562,7 @@
       </c>
       <c r="M883" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N883" s="4" t="inlineStr">
@@ -56690,7 +56690,7 @@
       </c>
       <c r="M885" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N885" s="4" t="inlineStr">
@@ -56754,7 +56754,7 @@
       </c>
       <c r="M886" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N886" s="4" t="inlineStr">
@@ -57010,7 +57010,7 @@
       </c>
       <c r="M890" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N890" s="4" t="inlineStr">
@@ -57138,7 +57138,7 @@
       </c>
       <c r="M892" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N892" s="4" t="inlineStr">
@@ -57394,7 +57394,7 @@
       </c>
       <c r="M896" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N896" s="4" t="inlineStr">
@@ -57522,7 +57522,7 @@
       </c>
       <c r="M898" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N898" s="4" t="inlineStr">
@@ -57586,7 +57586,7 @@
       </c>
       <c r="M899" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N899" s="4" t="inlineStr">
@@ -57714,7 +57714,7 @@
       </c>
       <c r="M901" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N901" s="4" t="inlineStr">
@@ -57970,7 +57970,7 @@
       </c>
       <c r="M905" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N905" s="4" t="inlineStr">
@@ -58290,7 +58290,7 @@
       </c>
       <c r="M910" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N910" s="4" t="inlineStr">
@@ -58482,7 +58482,7 @@
       </c>
       <c r="M913" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N913" s="4" t="inlineStr">
@@ -58990,7 +58990,7 @@
       </c>
       <c r="M921" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N921" s="4" t="inlineStr">
@@ -59118,7 +59118,7 @@
       </c>
       <c r="M923" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N923" s="4" t="inlineStr">
@@ -59182,7 +59182,7 @@
       </c>
       <c r="M924" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N924" s="4" t="inlineStr">
@@ -59246,7 +59246,7 @@
       </c>
       <c r="M925" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N925" s="4" t="inlineStr">
@@ -59310,7 +59310,7 @@
       </c>
       <c r="M926" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N926" s="4" t="inlineStr">
@@ -59374,7 +59374,7 @@
       </c>
       <c r="M927" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N927" s="4" t="inlineStr">
@@ -59438,7 +59438,7 @@
       </c>
       <c r="M928" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N928" s="4" t="inlineStr">
@@ -59502,7 +59502,7 @@
       </c>
       <c r="M929" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N929" s="4" t="inlineStr">
@@ -59758,7 +59758,7 @@
       </c>
       <c r="M933" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N933" s="4" t="inlineStr">
@@ -59822,7 +59822,7 @@
       </c>
       <c r="M934" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N934" s="4" t="inlineStr">
@@ -59950,7 +59950,7 @@
       </c>
       <c r="M936" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N936" s="4" t="inlineStr">
@@ -60014,7 +60014,7 @@
       </c>
       <c r="M937" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N937" s="4" t="inlineStr">
@@ -60078,7 +60078,7 @@
       </c>
       <c r="M938" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N938" s="4" t="inlineStr">
@@ -60202,7 +60202,7 @@
       </c>
       <c r="M940" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N940" s="4" t="inlineStr">
@@ -60330,7 +60330,7 @@
       </c>
       <c r="M942" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N942" s="4" t="inlineStr">
@@ -60522,7 +60522,7 @@
       </c>
       <c r="M945" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N945" s="4" t="inlineStr">
@@ -60778,7 +60778,7 @@
       </c>
       <c r="M949" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N949" s="4" t="inlineStr">
@@ -60842,7 +60842,7 @@
       </c>
       <c r="M950" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N950" s="4" t="inlineStr">
@@ -60906,7 +60906,7 @@
       </c>
       <c r="M951" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N951" s="4" t="inlineStr">
@@ -61034,7 +61034,7 @@
       </c>
       <c r="M953" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N953" s="4" t="inlineStr">
@@ -61098,7 +61098,7 @@
       </c>
       <c r="M954" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N954" s="4" t="inlineStr">
@@ -61290,7 +61290,7 @@
       </c>
       <c r="M957" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N957" s="4" t="inlineStr">
@@ -61610,7 +61610,7 @@
       </c>
       <c r="M962" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N962" s="4" t="inlineStr">
@@ -61866,7 +61866,7 @@
       </c>
       <c r="M966" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N966" s="4" t="inlineStr">
@@ -61930,7 +61930,7 @@
       </c>
       <c r="M967" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N967" s="4" t="inlineStr">
@@ -61994,7 +61994,7 @@
       </c>
       <c r="M968" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N968" s="4" t="inlineStr">
@@ -62058,7 +62058,7 @@
       </c>
       <c r="M969" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N969" s="4" t="inlineStr">
@@ -62250,7 +62250,7 @@
       </c>
       <c r="M972" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N972" s="4" t="inlineStr">
@@ -62378,7 +62378,7 @@
       </c>
       <c r="M974" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N974" s="4" t="inlineStr">
@@ -62570,7 +62570,7 @@
       </c>
       <c r="M977" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N977" s="4" t="inlineStr">
@@ -62826,7 +62826,7 @@
       </c>
       <c r="M981" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N981" s="4" t="inlineStr">
@@ -62890,7 +62890,7 @@
       </c>
       <c r="M982" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N982" s="4" t="inlineStr">
@@ -62954,7 +62954,7 @@
       </c>
       <c r="M983" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N983" s="4" t="inlineStr">
@@ -63078,7 +63078,7 @@
       </c>
       <c r="M985" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N985" s="4" t="inlineStr">
@@ -63206,7 +63206,7 @@
       </c>
       <c r="M987" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N987" s="4" t="inlineStr">
@@ -63526,7 +63526,7 @@
       </c>
       <c r="M992" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N992" s="4" t="inlineStr">
@@ -63846,7 +63846,7 @@
       </c>
       <c r="M997" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N997" s="4" t="inlineStr">
@@ -63906,7 +63906,7 @@
       </c>
       <c r="M998" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N998" s="4" t="inlineStr">
@@ -64098,7 +64098,7 @@
       </c>
       <c r="M1001" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1001" s="4" t="inlineStr">
@@ -64482,7 +64482,7 @@
       </c>
       <c r="M1007" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1007" s="4" t="inlineStr">
@@ -64546,7 +64546,7 @@
       </c>
       <c r="M1008" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1008" s="4" t="inlineStr">
@@ -64674,7 +64674,7 @@
       </c>
       <c r="M1010" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1010" s="4" t="inlineStr">
@@ -64738,7 +64738,7 @@
       </c>
       <c r="M1011" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1011" s="4" t="inlineStr">
@@ -64798,7 +64798,7 @@
       </c>
       <c r="M1012" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1012" s="4" t="inlineStr">
@@ -64862,7 +64862,7 @@
       </c>
       <c r="M1013" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1013" s="4" t="inlineStr">
@@ -65054,7 +65054,7 @@
       </c>
       <c r="M1016" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1016" s="4" t="inlineStr">
@@ -65246,7 +65246,7 @@
       </c>
       <c r="M1019" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1019" s="4" t="inlineStr">
@@ -65310,7 +65310,7 @@
       </c>
       <c r="M1020" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1020" s="4" t="inlineStr">
@@ -65694,7 +65694,7 @@
       </c>
       <c r="M1026" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1026" s="4" t="inlineStr">
@@ -65758,7 +65758,7 @@
       </c>
       <c r="M1027" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1027" s="4" t="inlineStr">
@@ -65886,7 +65886,7 @@
       </c>
       <c r="M1029" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1029" s="4" t="inlineStr">
@@ -65950,7 +65950,7 @@
       </c>
       <c r="M1030" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1030" s="4" t="inlineStr">
@@ -66014,7 +66014,7 @@
       </c>
       <c r="M1031" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1031" s="4" t="inlineStr">
@@ -66270,7 +66270,7 @@
       </c>
       <c r="M1035" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1035" s="4" t="inlineStr">
@@ -66334,7 +66334,7 @@
       </c>
       <c r="M1036" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1036" s="4" t="inlineStr">
@@ -66398,7 +66398,7 @@
       </c>
       <c r="M1037" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1037" s="4" t="inlineStr">
@@ -66462,7 +66462,7 @@
       </c>
       <c r="M1038" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1038" s="4" t="inlineStr">
@@ -66718,7 +66718,7 @@
       </c>
       <c r="M1042" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1042" s="4" t="inlineStr">
@@ -66910,7 +66910,7 @@
       </c>
       <c r="M1045" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1045" s="4" t="inlineStr">
@@ -66974,7 +66974,7 @@
       </c>
       <c r="M1046" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1046" s="4" t="inlineStr">
@@ -67102,7 +67102,7 @@
       </c>
       <c r="M1048" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1048" s="4" t="inlineStr">
@@ -67166,7 +67166,7 @@
       </c>
       <c r="M1049" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1049" s="4" t="inlineStr">
@@ -67230,7 +67230,7 @@
       </c>
       <c r="M1050" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1050" s="4" t="inlineStr">
@@ -67358,7 +67358,7 @@
       </c>
       <c r="M1052" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1052" s="4" t="inlineStr">
@@ -67422,7 +67422,7 @@
       </c>
       <c r="M1053" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1053" s="4" t="inlineStr">
@@ -67610,7 +67610,7 @@
       </c>
       <c r="M1056" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1056" s="4" t="inlineStr">
@@ -67738,7 +67738,7 @@
       </c>
       <c r="M1058" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1058" s="4" t="inlineStr">
@@ -67930,7 +67930,7 @@
       </c>
       <c r="M1061" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1061" s="4" t="inlineStr">
@@ -68118,7 +68118,7 @@
       </c>
       <c r="M1064" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1064" s="4" t="inlineStr">
@@ -68182,7 +68182,7 @@
       </c>
       <c r="M1065" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1065" s="4" t="inlineStr">
@@ -68246,7 +68246,7 @@
       </c>
       <c r="M1066" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1066" s="4" t="inlineStr">
@@ -68374,7 +68374,7 @@
       </c>
       <c r="M1068" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1068" s="4" t="inlineStr">
@@ -68498,7 +68498,7 @@
       </c>
       <c r="M1070" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1070" s="4" t="inlineStr">
@@ -68622,7 +68622,7 @@
       </c>
       <c r="M1072" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1072" s="4" t="inlineStr">
@@ -68750,7 +68750,7 @@
       </c>
       <c r="M1074" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1074" s="4" t="inlineStr">
@@ -68814,7 +68814,7 @@
       </c>
       <c r="M1075" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1075" s="4" t="inlineStr">
@@ -69378,7 +69378,7 @@
       </c>
       <c r="M1084" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1084" s="4" t="inlineStr">
@@ -69506,7 +69506,7 @@
       </c>
       <c r="M1086" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1086" s="4" t="inlineStr">
@@ -69570,7 +69570,7 @@
       </c>
       <c r="M1087" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1087" s="4" t="inlineStr">
@@ -69630,7 +69630,7 @@
       </c>
       <c r="M1088" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1088" s="4" t="inlineStr">
@@ -69690,7 +69690,7 @@
       </c>
       <c r="M1089" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1089" s="4" t="inlineStr">
@@ -69754,7 +69754,7 @@
       </c>
       <c r="M1090" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1090" s="4" t="inlineStr">
@@ -69818,7 +69818,7 @@
       </c>
       <c r="M1091" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1091" s="4" t="inlineStr">
@@ -69882,7 +69882,7 @@
       </c>
       <c r="M1092" s="4" t="inlineStr">
         <is>
-          <t>Ellikon an der Thur (Kellermann Gemüsekulturen)</t>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
         </is>
       </c>
       <c r="N1092" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Faktencheck eingearbeitet: Imhof in Hauptbetrieb/Gewächshaus geteilt, Bio-Status «unklar», Gerber-Angaben präzisiert, Legende nach Betrieb gruppiert
- config: Imhof-Teile nach Betriebsnummer (ZH0197/ 1/702 = Gewächshaus Eichhof, Betreiber und Bio offen);
  Gerber Bio Greens / Gemüsebau mit geprüften Orten und Bio-Angaben; Beerstecher ÖLN, Swiss GAP
- common.py: Bio-Code «offen» -> Status «Bio-Status unklar», Prüfung der Bio-Codes beim Laden
- Website: vierte Bio-Stufe (grau), Legende je Betrieb gruppiert (Name schaltet den ganzen Betrieb),
  Info-Texte zu Teilbetrieben und Gewächshäusern ohne Programm (ZH)
- docs/betriebe.md: Befunde und Quellen je Betrieb; Wohnadresse aus betriebsname entfernt
- Vorschaubild neu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQ5MKVLWHBWiVwJge7L58K
</commit_message>
<xml_diff>
--- a/output/Feldkarte_Flaechen_4_Betriebe.xlsx
+++ b/output/Feldkarte_Flaechen_4_Betriebe.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -500,7 +500,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Betriebsnummern: Imhof ZH0197/ 1/  1 + ZH0197/ 1/702 · Beerstecher ZH0191/ 1/ 55 · Gerber ZH0172/ 1/700 (Zwei Firmen unter einer Betriebsnummer; aufgeteilt nach den amtlichen Produktionsstätten) · Rathgeb ZH0042/ 1/850 + TG39621 (Unternehmensgruppe: drei Teile unter zwei Betriebsnummern, getrennt nach amtlicher Produktionsstätte)</t>
+          <t>Betriebsnummern: Imhof ZH0197/ 1/  1 + ZH0197/ 1/702 (Zwei Betriebsnummern auf dem Eichhof, getrennt nach Betriebsnummer) · Beerstecher ZH0191/ 1/ 55 · Gerber ZH0172/ 1/700 (Zwei Firmen unter einer Betriebsnummer, getrennt nach amtlicher Produktionsstätte (Firma über die Adresse zugeordnet)) · Rathgeb ZH0042/ 1/850 + TG39621 (Unternehmensgruppe: drei Teile unter zwei Betriebsnummern, getrennt nach amtlicher Produktionsstätte)</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Teilbetriebe (aufgeteilt nach amtlicher Produktionsstätte)</t>
+          <t>Teilbetriebe (aufgeteilt nach Betriebsnummer bzw. amtlicher Produktionsstätte)</t>
         </is>
       </c>
     </row>
@@ -875,123 +875,123 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Gerber Bio Greens AG</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Gerber</t>
+          <t>Imhof</t>
         </is>
       </c>
       <c r="C20" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A20)</f>
-        <v>106.073</v>
+        <v>90.609</v>
       </c>
       <c r="D20" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A20,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A20,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
-        <v>60.86</v>
+        <v>45.287</v>
       </c>
       <c r="E20" s="4">
         <f>COUNTIF(Flächen!$M$2:$M$1093,$A20)</f>
-        <v>161</v>
+        <v>245</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Bio (Knospe) laut Firma; in den Kantonsdaten nicht als Bio gemeldet</t>
+          <t>Bio Suisse (Knospe), Gemüse nach Demeter; Flächen 2025 als Bioproduktion gemeldet</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Gerber Gemüsebau AG</t>
+          <t>Gewächshaus Eichhof</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Gerber</t>
+          <t>Imhof</t>
         </is>
       </c>
       <c r="C21" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A21)</f>
-        <v>147.079</v>
+        <v>1.019</v>
       </c>
       <c r="D21" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A21,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A21,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
-        <v>138.096</v>
+        <v>1.019</v>
       </c>
       <c r="E21" s="4">
         <f>COUNTIF(Flächen!$M$2:$M$1093,$A21)</f>
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>konventionell (Suisse Garantie)</t>
+          <t>Bio-Status unklar: Gewächshäuser mit festem Fundament tragen in den Zürcher Daten nie ein Programm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Rathgeb Bio, Unterstammheim</t>
+          <t>Gerber Bio Greens AG</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Rathgeb</t>
+          <t>Gerber</t>
         </is>
       </c>
       <c r="C22" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A22)</f>
-        <v>289.053</v>
+        <v>106.073</v>
       </c>
       <c r="D22" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A22,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A22,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
-        <v>144.966</v>
+        <v>60.86</v>
       </c>
       <c r="E22" s="4">
         <f>COUNTIF(Flächen!$M$2:$M$1093,$A22)</f>
-        <v>228</v>
+        <v>161</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
+          <t>Bio Suisse (Knospe) laut Firma; 2025 keine Fläche als Bioproduktion gemeldet</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Rathgeb Bio, Ellikon an der Thur</t>
+          <t>Gerber Gemüsebau AG</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Rathgeb</t>
+          <t>Gerber</t>
         </is>
       </c>
       <c r="C23" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A23)</f>
-        <v>253.068</v>
+        <v>147.079</v>
       </c>
       <c r="D23" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A23,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A23,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
-        <v>136.268</v>
+        <v>138.096</v>
       </c>
       <c r="E23" s="4">
         <f>COUNTIF(Flächen!$M$2:$M$1093,$A23)</f>
-        <v>201</v>
+        <v>71</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
+          <t>konventionell, Suisse Garantie (laut Firma)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>BioFresh AG, Tägerwilen</t>
+          <t>Rathgeb Bio, Unterstammheim</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1001,17 +1001,75 @@
       </c>
       <c r="C24" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A24)</f>
-        <v>8.185</v>
+        <v>289.053</v>
       </c>
       <c r="D24" s="5">
         <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A24,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A24,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
-        <v>7.478</v>
+        <v>144.966</v>
       </c>
       <c r="E24" s="4">
         <f>COUNTIF(Flächen!$M$2:$M$1093,$A24)</f>
+        <v>228</v>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Rathgeb Bio, Ellikon an der Thur</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Rathgeb</t>
+        </is>
+      </c>
+      <c r="C25" s="5">
+        <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A25)</f>
+        <v>253.068</v>
+      </c>
+      <c r="D25" s="5">
+        <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A25,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A25,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
+        <v>136.268</v>
+      </c>
+      <c r="E25" s="4">
+        <f>COUNTIF(Flächen!$M$2:$M$1093,$A25)</f>
+        <v>201</v>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>BioFresh AG, Tägerwilen</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Rathgeb</t>
+        </is>
+      </c>
+      <c r="C26" s="5">
+        <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A26)</f>
+        <v>8.185</v>
+      </c>
+      <c r="D26" s="5">
+        <f>SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A26,Flächen!$E$2:$E$1093,"Freilandgemüse")+SUMIFS(Flächen!$G$2:$G$1093,Flächen!$M$2:$M$1093,$A26,Flächen!$E$2:$E$1093,"Gewächshaus / geschützt")</f>
+        <v>7.478</v>
+      </c>
+      <c r="E26" s="4">
+        <f>COUNTIF(Flächen!$M$2:$M$1093,$A26)</f>
         <v>12</v>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Bio Suisse (Knospe); Flächen 2025 als Bioproduktion gemeldet</t>
         </is>
@@ -26214,7 +26272,7 @@
       </c>
       <c r="M407" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N407" s="4" t="inlineStr">
@@ -26278,7 +26336,7 @@
       </c>
       <c r="M408" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N408" s="4" t="inlineStr">
@@ -26342,7 +26400,7 @@
       </c>
       <c r="M409" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N409" s="4" t="inlineStr">
@@ -26406,7 +26464,7 @@
       </c>
       <c r="M410" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N410" s="4" t="inlineStr">
@@ -26470,7 +26528,7 @@
       </c>
       <c r="M411" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N411" s="4" t="inlineStr">
@@ -26534,7 +26592,7 @@
       </c>
       <c r="M412" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N412" s="4" t="inlineStr">
@@ -26598,7 +26656,7 @@
       </c>
       <c r="M413" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N413" s="4" t="inlineStr">
@@ -26662,7 +26720,7 @@
       </c>
       <c r="M414" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N414" s="4" t="inlineStr">
@@ -26726,7 +26784,7 @@
       </c>
       <c r="M415" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N415" s="4" t="inlineStr">
@@ -26790,7 +26848,7 @@
       </c>
       <c r="M416" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N416" s="4" t="inlineStr">
@@ -26854,7 +26912,7 @@
       </c>
       <c r="M417" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N417" s="4" t="inlineStr">
@@ -26918,7 +26976,7 @@
       </c>
       <c r="M418" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N418" s="4" t="inlineStr">
@@ -26982,7 +27040,7 @@
       </c>
       <c r="M419" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N419" s="4" t="inlineStr">
@@ -27042,7 +27100,7 @@
       </c>
       <c r="M420" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N420" s="4" t="inlineStr">
@@ -27106,7 +27164,7 @@
       </c>
       <c r="M421" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N421" s="4" t="inlineStr">
@@ -27170,7 +27228,7 @@
       </c>
       <c r="M422" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N422" s="4" t="inlineStr">
@@ -27234,7 +27292,7 @@
       </c>
       <c r="M423" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N423" s="4" t="inlineStr">
@@ -27298,7 +27356,7 @@
       </c>
       <c r="M424" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N424" s="4" t="inlineStr">
@@ -27362,7 +27420,7 @@
       </c>
       <c r="M425" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N425" s="4" t="inlineStr">
@@ -27426,7 +27484,7 @@
       </c>
       <c r="M426" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N426" s="4" t="inlineStr">
@@ -27490,7 +27548,7 @@
       </c>
       <c r="M427" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N427" s="4" t="inlineStr">
@@ -27554,7 +27612,7 @@
       </c>
       <c r="M428" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N428" s="4" t="inlineStr">
@@ -27618,7 +27676,7 @@
       </c>
       <c r="M429" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N429" s="4" t="inlineStr">
@@ -27682,7 +27740,7 @@
       </c>
       <c r="M430" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N430" s="4" t="inlineStr">
@@ -27746,7 +27804,7 @@
       </c>
       <c r="M431" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N431" s="4" t="inlineStr">
@@ -27806,12 +27864,12 @@
       </c>
       <c r="M432" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Gewächshaus Eichhof</t>
         </is>
       </c>
       <c r="N432" s="4" t="inlineStr">
         <is>
-          <t>Bio-Betrieb, Fläche nicht als Bio gemeldet</t>
+          <t>Bio-Status unklar</t>
         </is>
       </c>
     </row>
@@ -27870,7 +27928,7 @@
       </c>
       <c r="M433" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N433" s="4" t="inlineStr">
@@ -27934,7 +27992,7 @@
       </c>
       <c r="M434" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N434" s="4" t="inlineStr">
@@ -27998,7 +28056,7 @@
       </c>
       <c r="M435" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N435" s="4" t="inlineStr">
@@ -28062,7 +28120,7 @@
       </c>
       <c r="M436" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N436" s="4" t="inlineStr">
@@ -28126,7 +28184,7 @@
       </c>
       <c r="M437" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N437" s="4" t="inlineStr">
@@ -28190,7 +28248,7 @@
       </c>
       <c r="M438" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N438" s="4" t="inlineStr">
@@ -28254,7 +28312,7 @@
       </c>
       <c r="M439" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N439" s="4" t="inlineStr">
@@ -28318,7 +28376,7 @@
       </c>
       <c r="M440" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N440" s="4" t="inlineStr">
@@ -28378,7 +28436,7 @@
       </c>
       <c r="M441" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N441" s="4" t="inlineStr">
@@ -28442,7 +28500,7 @@
       </c>
       <c r="M442" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N442" s="4" t="inlineStr">
@@ -28506,7 +28564,7 @@
       </c>
       <c r="M443" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N443" s="4" t="inlineStr">
@@ -28570,7 +28628,7 @@
       </c>
       <c r="M444" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N444" s="4" t="inlineStr">
@@ -28634,7 +28692,7 @@
       </c>
       <c r="M445" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N445" s="4" t="inlineStr">
@@ -28698,7 +28756,7 @@
       </c>
       <c r="M446" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N446" s="4" t="inlineStr">
@@ -28762,7 +28820,7 @@
       </c>
       <c r="M447" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N447" s="4" t="inlineStr">
@@ -28826,7 +28884,7 @@
       </c>
       <c r="M448" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N448" s="4" t="inlineStr">
@@ -28890,7 +28948,7 @@
       </c>
       <c r="M449" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N449" s="4" t="inlineStr">
@@ -28954,7 +29012,7 @@
       </c>
       <c r="M450" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N450" s="4" t="inlineStr">
@@ -29018,7 +29076,7 @@
       </c>
       <c r="M451" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N451" s="4" t="inlineStr">
@@ -29082,7 +29140,7 @@
       </c>
       <c r="M452" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N452" s="4" t="inlineStr">
@@ -29146,7 +29204,7 @@
       </c>
       <c r="M453" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N453" s="4" t="inlineStr">
@@ -29210,7 +29268,7 @@
       </c>
       <c r="M454" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N454" s="4" t="inlineStr">
@@ -29274,7 +29332,7 @@
       </c>
       <c r="M455" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N455" s="4" t="inlineStr">
@@ -29338,7 +29396,7 @@
       </c>
       <c r="M456" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N456" s="4" t="inlineStr">
@@ -29402,7 +29460,7 @@
       </c>
       <c r="M457" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N457" s="4" t="inlineStr">
@@ -29466,7 +29524,7 @@
       </c>
       <c r="M458" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N458" s="4" t="inlineStr">
@@ -29530,7 +29588,7 @@
       </c>
       <c r="M459" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N459" s="4" t="inlineStr">
@@ -29590,7 +29648,7 @@
       </c>
       <c r="M460" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N460" s="4" t="inlineStr">
@@ -29654,7 +29712,7 @@
       </c>
       <c r="M461" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N461" s="4" t="inlineStr">
@@ -29718,7 +29776,7 @@
       </c>
       <c r="M462" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N462" s="4" t="inlineStr">
@@ -29778,7 +29836,7 @@
       </c>
       <c r="M463" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N463" s="4" t="inlineStr">
@@ -29842,7 +29900,7 @@
       </c>
       <c r="M464" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N464" s="4" t="inlineStr">
@@ -29906,7 +29964,7 @@
       </c>
       <c r="M465" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N465" s="4" t="inlineStr">
@@ -29970,7 +30028,7 @@
       </c>
       <c r="M466" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N466" s="4" t="inlineStr">
@@ -30034,7 +30092,7 @@
       </c>
       <c r="M467" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N467" s="4" t="inlineStr">
@@ -30098,7 +30156,7 @@
       </c>
       <c r="M468" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N468" s="4" t="inlineStr">
@@ -30162,7 +30220,7 @@
       </c>
       <c r="M469" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N469" s="4" t="inlineStr">
@@ -30226,7 +30284,7 @@
       </c>
       <c r="M470" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N470" s="4" t="inlineStr">
@@ -30290,7 +30348,7 @@
       </c>
       <c r="M471" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N471" s="4" t="inlineStr">
@@ -30354,7 +30412,7 @@
       </c>
       <c r="M472" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N472" s="4" t="inlineStr">
@@ -30418,7 +30476,7 @@
       </c>
       <c r="M473" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N473" s="4" t="inlineStr">
@@ -30482,7 +30540,7 @@
       </c>
       <c r="M474" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N474" s="4" t="inlineStr">
@@ -30546,7 +30604,7 @@
       </c>
       <c r="M475" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N475" s="4" t="inlineStr">
@@ -30610,7 +30668,7 @@
       </c>
       <c r="M476" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N476" s="4" t="inlineStr">
@@ -30674,7 +30732,7 @@
       </c>
       <c r="M477" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N477" s="4" t="inlineStr">
@@ -30738,7 +30796,7 @@
       </c>
       <c r="M478" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N478" s="4" t="inlineStr">
@@ -30802,7 +30860,7 @@
       </c>
       <c r="M479" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N479" s="4" t="inlineStr">
@@ -30866,7 +30924,7 @@
       </c>
       <c r="M480" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N480" s="4" t="inlineStr">
@@ -30930,7 +30988,7 @@
       </c>
       <c r="M481" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N481" s="4" t="inlineStr">
@@ -30994,7 +31052,7 @@
       </c>
       <c r="M482" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N482" s="4" t="inlineStr">
@@ -31058,7 +31116,7 @@
       </c>
       <c r="M483" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N483" s="4" t="inlineStr">
@@ -31122,7 +31180,7 @@
       </c>
       <c r="M484" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N484" s="4" t="inlineStr">
@@ -31186,7 +31244,7 @@
       </c>
       <c r="M485" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N485" s="4" t="inlineStr">
@@ -31250,7 +31308,7 @@
       </c>
       <c r="M486" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N486" s="4" t="inlineStr">
@@ -31314,7 +31372,7 @@
       </c>
       <c r="M487" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N487" s="4" t="inlineStr">
@@ -31378,7 +31436,7 @@
       </c>
       <c r="M488" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N488" s="4" t="inlineStr">
@@ -31442,7 +31500,7 @@
       </c>
       <c r="M489" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N489" s="4" t="inlineStr">
@@ -31506,7 +31564,7 @@
       </c>
       <c r="M490" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N490" s="4" t="inlineStr">
@@ -31570,7 +31628,7 @@
       </c>
       <c r="M491" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N491" s="4" t="inlineStr">
@@ -31634,7 +31692,7 @@
       </c>
       <c r="M492" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N492" s="4" t="inlineStr">
@@ -31698,7 +31756,7 @@
       </c>
       <c r="M493" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N493" s="4" t="inlineStr">
@@ -31762,7 +31820,7 @@
       </c>
       <c r="M494" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N494" s="4" t="inlineStr">
@@ -31822,7 +31880,7 @@
       </c>
       <c r="M495" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N495" s="4" t="inlineStr">
@@ -31882,7 +31940,7 @@
       </c>
       <c r="M496" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N496" s="4" t="inlineStr">
@@ -31942,7 +32000,7 @@
       </c>
       <c r="M497" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N497" s="4" t="inlineStr">
@@ -32006,7 +32064,7 @@
       </c>
       <c r="M498" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N498" s="4" t="inlineStr">
@@ -32070,7 +32128,7 @@
       </c>
       <c r="M499" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N499" s="4" t="inlineStr">
@@ -32134,7 +32192,7 @@
       </c>
       <c r="M500" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N500" s="4" t="inlineStr">
@@ -32198,7 +32256,7 @@
       </c>
       <c r="M501" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N501" s="4" t="inlineStr">
@@ -32262,7 +32320,7 @@
       </c>
       <c r="M502" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N502" s="4" t="inlineStr">
@@ -32326,7 +32384,7 @@
       </c>
       <c r="M503" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N503" s="4" t="inlineStr">
@@ -32390,7 +32448,7 @@
       </c>
       <c r="M504" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N504" s="4" t="inlineStr">
@@ -32454,7 +32512,7 @@
       </c>
       <c r="M505" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N505" s="4" t="inlineStr">
@@ -32518,7 +32576,7 @@
       </c>
       <c r="M506" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N506" s="4" t="inlineStr">
@@ -32582,7 +32640,7 @@
       </c>
       <c r="M507" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N507" s="4" t="inlineStr">
@@ -32646,7 +32704,7 @@
       </c>
       <c r="M508" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N508" s="4" t="inlineStr">
@@ -32710,7 +32768,7 @@
       </c>
       <c r="M509" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N509" s="4" t="inlineStr">
@@ -32770,7 +32828,7 @@
       </c>
       <c r="M510" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N510" s="4" t="inlineStr">
@@ -32834,7 +32892,7 @@
       </c>
       <c r="M511" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N511" s="4" t="inlineStr">
@@ -32898,7 +32956,7 @@
       </c>
       <c r="M512" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N512" s="4" t="inlineStr">
@@ -32962,7 +33020,7 @@
       </c>
       <c r="M513" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N513" s="4" t="inlineStr">
@@ -33026,7 +33084,7 @@
       </c>
       <c r="M514" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N514" s="4" t="inlineStr">
@@ -33090,7 +33148,7 @@
       </c>
       <c r="M515" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N515" s="4" t="inlineStr">
@@ -33154,7 +33212,7 @@
       </c>
       <c r="M516" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N516" s="4" t="inlineStr">
@@ -33218,7 +33276,7 @@
       </c>
       <c r="M517" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N517" s="4" t="inlineStr">
@@ -33282,7 +33340,7 @@
       </c>
       <c r="M518" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N518" s="4" t="inlineStr">
@@ -33342,7 +33400,7 @@
       </c>
       <c r="M519" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N519" s="4" t="inlineStr">
@@ -33406,7 +33464,7 @@
       </c>
       <c r="M520" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N520" s="4" t="inlineStr">
@@ -33470,7 +33528,7 @@
       </c>
       <c r="M521" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N521" s="4" t="inlineStr">
@@ -33534,7 +33592,7 @@
       </c>
       <c r="M522" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N522" s="4" t="inlineStr">
@@ -33598,7 +33656,7 @@
       </c>
       <c r="M523" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N523" s="4" t="inlineStr">
@@ -33662,7 +33720,7 @@
       </c>
       <c r="M524" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N524" s="4" t="inlineStr">
@@ -33726,7 +33784,7 @@
       </c>
       <c r="M525" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N525" s="4" t="inlineStr">
@@ -33790,7 +33848,7 @@
       </c>
       <c r="M526" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N526" s="4" t="inlineStr">
@@ -33854,7 +33912,7 @@
       </c>
       <c r="M527" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N527" s="4" t="inlineStr">
@@ -33918,7 +33976,7 @@
       </c>
       <c r="M528" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N528" s="4" t="inlineStr">
@@ -33982,7 +34040,7 @@
       </c>
       <c r="M529" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N529" s="4" t="inlineStr">
@@ -34046,7 +34104,7 @@
       </c>
       <c r="M530" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N530" s="4" t="inlineStr">
@@ -34110,7 +34168,7 @@
       </c>
       <c r="M531" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N531" s="4" t="inlineStr">
@@ -34174,7 +34232,7 @@
       </c>
       <c r="M532" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N532" s="4" t="inlineStr">
@@ -34234,7 +34292,7 @@
       </c>
       <c r="M533" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N533" s="4" t="inlineStr">
@@ -34298,7 +34356,7 @@
       </c>
       <c r="M534" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N534" s="4" t="inlineStr">
@@ -34362,7 +34420,7 @@
       </c>
       <c r="M535" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N535" s="4" t="inlineStr">
@@ -34422,7 +34480,7 @@
       </c>
       <c r="M536" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N536" s="4" t="inlineStr">
@@ -34486,7 +34544,7 @@
       </c>
       <c r="M537" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N537" s="4" t="inlineStr">
@@ -34550,7 +34608,7 @@
       </c>
       <c r="M538" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N538" s="4" t="inlineStr">
@@ -34610,7 +34668,7 @@
       </c>
       <c r="M539" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N539" s="4" t="inlineStr">
@@ -34674,7 +34732,7 @@
       </c>
       <c r="M540" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N540" s="4" t="inlineStr">
@@ -34738,7 +34796,7 @@
       </c>
       <c r="M541" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N541" s="4" t="inlineStr">
@@ -34798,7 +34856,7 @@
       </c>
       <c r="M542" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N542" s="4" t="inlineStr">
@@ -34862,7 +34920,7 @@
       </c>
       <c r="M543" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N543" s="4" t="inlineStr">
@@ -34922,7 +34980,7 @@
       </c>
       <c r="M544" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N544" s="4" t="inlineStr">
@@ -34986,7 +35044,7 @@
       </c>
       <c r="M545" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N545" s="4" t="inlineStr">
@@ -35050,7 +35108,7 @@
       </c>
       <c r="M546" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N546" s="4" t="inlineStr">
@@ -35114,7 +35172,7 @@
       </c>
       <c r="M547" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N547" s="4" t="inlineStr">
@@ -35178,7 +35236,7 @@
       </c>
       <c r="M548" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N548" s="4" t="inlineStr">
@@ -35242,7 +35300,7 @@
       </c>
       <c r="M549" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N549" s="4" t="inlineStr">
@@ -35306,7 +35364,7 @@
       </c>
       <c r="M550" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N550" s="4" t="inlineStr">
@@ -35366,7 +35424,7 @@
       </c>
       <c r="M551" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N551" s="4" t="inlineStr">
@@ -35430,7 +35488,7 @@
       </c>
       <c r="M552" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N552" s="4" t="inlineStr">
@@ -35494,7 +35552,7 @@
       </c>
       <c r="M553" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N553" s="4" t="inlineStr">
@@ -35554,7 +35612,7 @@
       </c>
       <c r="M554" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N554" s="4" t="inlineStr">
@@ -35618,7 +35676,7 @@
       </c>
       <c r="M555" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N555" s="4" t="inlineStr">
@@ -35682,7 +35740,7 @@
       </c>
       <c r="M556" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N556" s="4" t="inlineStr">
@@ -35746,7 +35804,7 @@
       </c>
       <c r="M557" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N557" s="4" t="inlineStr">
@@ -35810,7 +35868,7 @@
       </c>
       <c r="M558" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N558" s="4" t="inlineStr">
@@ -35874,7 +35932,7 @@
       </c>
       <c r="M559" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N559" s="4" t="inlineStr">
@@ -35938,7 +35996,7 @@
       </c>
       <c r="M560" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N560" s="4" t="inlineStr">
@@ -36002,7 +36060,7 @@
       </c>
       <c r="M561" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N561" s="4" t="inlineStr">
@@ -36066,7 +36124,7 @@
       </c>
       <c r="M562" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N562" s="4" t="inlineStr">
@@ -36130,7 +36188,7 @@
       </c>
       <c r="M563" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N563" s="4" t="inlineStr">
@@ -36194,7 +36252,7 @@
       </c>
       <c r="M564" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N564" s="4" t="inlineStr">
@@ -36254,7 +36312,7 @@
       </c>
       <c r="M565" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N565" s="4" t="inlineStr">
@@ -36318,7 +36376,7 @@
       </c>
       <c r="M566" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N566" s="4" t="inlineStr">
@@ -36382,7 +36440,7 @@
       </c>
       <c r="M567" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N567" s="4" t="inlineStr">
@@ -36446,7 +36504,7 @@
       </c>
       <c r="M568" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N568" s="4" t="inlineStr">
@@ -36510,7 +36568,7 @@
       </c>
       <c r="M569" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N569" s="4" t="inlineStr">
@@ -36574,7 +36632,7 @@
       </c>
       <c r="M570" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N570" s="4" t="inlineStr">
@@ -36638,7 +36696,7 @@
       </c>
       <c r="M571" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N571" s="4" t="inlineStr">
@@ -36702,7 +36760,7 @@
       </c>
       <c r="M572" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N572" s="4" t="inlineStr">
@@ -36762,7 +36820,7 @@
       </c>
       <c r="M573" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N573" s="4" t="inlineStr">
@@ -36826,7 +36884,7 @@
       </c>
       <c r="M574" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N574" s="4" t="inlineStr">
@@ -36890,7 +36948,7 @@
       </c>
       <c r="M575" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N575" s="4" t="inlineStr">
@@ -36954,7 +37012,7 @@
       </c>
       <c r="M576" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N576" s="4" t="inlineStr">
@@ -37018,7 +37076,7 @@
       </c>
       <c r="M577" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N577" s="4" t="inlineStr">
@@ -37078,7 +37136,7 @@
       </c>
       <c r="M578" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N578" s="4" t="inlineStr">
@@ -37138,7 +37196,7 @@
       </c>
       <c r="M579" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N579" s="4" t="inlineStr">
@@ -37202,7 +37260,7 @@
       </c>
       <c r="M580" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N580" s="4" t="inlineStr">
@@ -37266,7 +37324,7 @@
       </c>
       <c r="M581" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N581" s="4" t="inlineStr">
@@ -37330,7 +37388,7 @@
       </c>
       <c r="M582" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N582" s="4" t="inlineStr">
@@ -37394,7 +37452,7 @@
       </c>
       <c r="M583" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N583" s="4" t="inlineStr">
@@ -37458,7 +37516,7 @@
       </c>
       <c r="M584" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N584" s="4" t="inlineStr">
@@ -37522,7 +37580,7 @@
       </c>
       <c r="M585" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N585" s="4" t="inlineStr">
@@ -37586,7 +37644,7 @@
       </c>
       <c r="M586" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N586" s="4" t="inlineStr">
@@ -37646,7 +37704,7 @@
       </c>
       <c r="M587" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N587" s="4" t="inlineStr">
@@ -37710,7 +37768,7 @@
       </c>
       <c r="M588" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N588" s="4" t="inlineStr">
@@ -37774,7 +37832,7 @@
       </c>
       <c r="M589" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N589" s="4" t="inlineStr">
@@ -37838,7 +37896,7 @@
       </c>
       <c r="M590" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N590" s="4" t="inlineStr">
@@ -37902,7 +37960,7 @@
       </c>
       <c r="M591" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N591" s="4" t="inlineStr">
@@ -37966,7 +38024,7 @@
       </c>
       <c r="M592" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N592" s="4" t="inlineStr">
@@ -38030,7 +38088,7 @@
       </c>
       <c r="M593" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N593" s="4" t="inlineStr">
@@ -38094,7 +38152,7 @@
       </c>
       <c r="M594" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N594" s="4" t="inlineStr">
@@ -38158,7 +38216,7 @@
       </c>
       <c r="M595" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N595" s="4" t="inlineStr">
@@ -38222,7 +38280,7 @@
       </c>
       <c r="M596" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N596" s="4" t="inlineStr">
@@ -38286,7 +38344,7 @@
       </c>
       <c r="M597" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N597" s="4" t="inlineStr">
@@ -38350,7 +38408,7 @@
       </c>
       <c r="M598" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N598" s="4" t="inlineStr">
@@ -38414,7 +38472,7 @@
       </c>
       <c r="M599" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N599" s="4" t="inlineStr">
@@ -38478,7 +38536,7 @@
       </c>
       <c r="M600" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N600" s="4" t="inlineStr">
@@ -38542,7 +38600,7 @@
       </c>
       <c r="M601" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N601" s="4" t="inlineStr">
@@ -38606,7 +38664,7 @@
       </c>
       <c r="M602" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N602" s="4" t="inlineStr">
@@ -38670,7 +38728,7 @@
       </c>
       <c r="M603" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N603" s="4" t="inlineStr">
@@ -38734,7 +38792,7 @@
       </c>
       <c r="M604" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N604" s="4" t="inlineStr">
@@ -38798,7 +38856,7 @@
       </c>
       <c r="M605" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N605" s="4" t="inlineStr">
@@ -38862,7 +38920,7 @@
       </c>
       <c r="M606" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N606" s="4" t="inlineStr">
@@ -38922,7 +38980,7 @@
       </c>
       <c r="M607" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N607" s="4" t="inlineStr">
@@ -38986,7 +39044,7 @@
       </c>
       <c r="M608" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N608" s="4" t="inlineStr">
@@ -39050,7 +39108,7 @@
       </c>
       <c r="M609" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N609" s="4" t="inlineStr">
@@ -39114,7 +39172,7 @@
       </c>
       <c r="M610" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N610" s="4" t="inlineStr">
@@ -39178,7 +39236,7 @@
       </c>
       <c r="M611" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N611" s="4" t="inlineStr">
@@ -39242,7 +39300,7 @@
       </c>
       <c r="M612" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N612" s="4" t="inlineStr">
@@ -39306,7 +39364,7 @@
       </c>
       <c r="M613" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N613" s="4" t="inlineStr">
@@ -39370,7 +39428,7 @@
       </c>
       <c r="M614" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N614" s="4" t="inlineStr">
@@ -39434,7 +39492,7 @@
       </c>
       <c r="M615" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N615" s="4" t="inlineStr">
@@ -39498,7 +39556,7 @@
       </c>
       <c r="M616" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N616" s="4" t="inlineStr">
@@ -39562,7 +39620,7 @@
       </c>
       <c r="M617" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N617" s="4" t="inlineStr">
@@ -39626,7 +39684,7 @@
       </c>
       <c r="M618" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N618" s="4" t="inlineStr">
@@ -39690,7 +39748,7 @@
       </c>
       <c r="M619" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N619" s="4" t="inlineStr">
@@ -39754,7 +39812,7 @@
       </c>
       <c r="M620" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N620" s="4" t="inlineStr">
@@ -39814,7 +39872,7 @@
       </c>
       <c r="M621" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N621" s="4" t="inlineStr">
@@ -39878,7 +39936,7 @@
       </c>
       <c r="M622" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N622" s="4" t="inlineStr">
@@ -39942,7 +40000,7 @@
       </c>
       <c r="M623" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N623" s="4" t="inlineStr">
@@ -40006,7 +40064,7 @@
       </c>
       <c r="M624" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N624" s="4" t="inlineStr">
@@ -40070,7 +40128,7 @@
       </c>
       <c r="M625" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N625" s="4" t="inlineStr">
@@ -40130,7 +40188,7 @@
       </c>
       <c r="M626" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N626" s="4" t="inlineStr">
@@ -40194,7 +40252,7 @@
       </c>
       <c r="M627" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N627" s="4" t="inlineStr">
@@ -40258,7 +40316,7 @@
       </c>
       <c r="M628" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N628" s="4" t="inlineStr">
@@ -40322,7 +40380,7 @@
       </c>
       <c r="M629" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N629" s="4" t="inlineStr">
@@ -40386,7 +40444,7 @@
       </c>
       <c r="M630" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N630" s="4" t="inlineStr">
@@ -40450,7 +40508,7 @@
       </c>
       <c r="M631" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N631" s="4" t="inlineStr">
@@ -40514,7 +40572,7 @@
       </c>
       <c r="M632" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N632" s="4" t="inlineStr">
@@ -40578,7 +40636,7 @@
       </c>
       <c r="M633" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N633" s="4" t="inlineStr">
@@ -40642,7 +40700,7 @@
       </c>
       <c r="M634" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N634" s="4" t="inlineStr">
@@ -40706,7 +40764,7 @@
       </c>
       <c r="M635" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N635" s="4" t="inlineStr">
@@ -40770,7 +40828,7 @@
       </c>
       <c r="M636" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N636" s="4" t="inlineStr">
@@ -40834,7 +40892,7 @@
       </c>
       <c r="M637" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N637" s="4" t="inlineStr">
@@ -40898,7 +40956,7 @@
       </c>
       <c r="M638" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N638" s="4" t="inlineStr">
@@ -40962,7 +41020,7 @@
       </c>
       <c r="M639" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N639" s="4" t="inlineStr">
@@ -41026,7 +41084,7 @@
       </c>
       <c r="M640" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N640" s="4" t="inlineStr">
@@ -41086,7 +41144,7 @@
       </c>
       <c r="M641" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N641" s="4" t="inlineStr">
@@ -41150,7 +41208,7 @@
       </c>
       <c r="M642" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N642" s="4" t="inlineStr">
@@ -41214,7 +41272,7 @@
       </c>
       <c r="M643" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N643" s="4" t="inlineStr">
@@ -41278,7 +41336,7 @@
       </c>
       <c r="M644" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N644" s="4" t="inlineStr">
@@ -41342,7 +41400,7 @@
       </c>
       <c r="M645" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N645" s="4" t="inlineStr">
@@ -41406,7 +41464,7 @@
       </c>
       <c r="M646" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N646" s="4" t="inlineStr">
@@ -41470,7 +41528,7 @@
       </c>
       <c r="M647" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N647" s="4" t="inlineStr">
@@ -41534,7 +41592,7 @@
       </c>
       <c r="M648" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N648" s="4" t="inlineStr">
@@ -41598,7 +41656,7 @@
       </c>
       <c r="M649" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N649" s="4" t="inlineStr">
@@ -41662,7 +41720,7 @@
       </c>
       <c r="M650" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N650" s="4" t="inlineStr">
@@ -41726,7 +41784,7 @@
       </c>
       <c r="M651" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N651" s="4" t="inlineStr">
@@ -41786,7 +41844,7 @@
       </c>
       <c r="M652" s="4" t="inlineStr">
         <is>
-          <t>Imhof</t>
+          <t>Imhofbio, Eichhof Schwerzenbach</t>
         </is>
       </c>
       <c r="N652" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Imhof: ZH0197/ 1/702 ist die Imhof Flora AG (Angabe Alex), nicht Bio
Website, Excel, GeoPackage, PDF-Übersicht und Doku nachgeführt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQ5MKVLWHBWiVwJge7L58K
</commit_message>
<xml_diff>
--- a/output/Feldkarte_Flaechen_4_Betriebe.xlsx
+++ b/output/Feldkarte_Flaechen_4_Betriebe.xlsx
@@ -916,7 +916,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Gewächshaus Eichhof</t>
+          <t>Imhof Flora AG</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>Bio-Status unklar: Gewächshäuser mit festem Fundament tragen in den Zürcher Daten nie ein Programm</t>
+          <t>nicht Bio (Swiss GAP, Suisse Garantie)</t>
         </is>
       </c>
     </row>
@@ -27900,12 +27900,12 @@
       </c>
       <c r="M432" s="4" t="inlineStr">
         <is>
-          <t>Gewächshaus Eichhof</t>
+          <t>Imhof Flora AG</t>
         </is>
       </c>
       <c r="N432" s="4" t="inlineStr">
         <is>
-          <t>Bio-Status unklar</t>
+          <t>nicht Bio</t>
         </is>
       </c>
     </row>

</xml_diff>